<commit_message>
Update Excel sheet with recovered changes
</commit_message>
<xml_diff>
--- a/IT23665866_Assignment 1 - Test cases.xlsx
+++ b/IT23665866_Assignment 1 - Test cases.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Novaline\Downloads\IT23665866\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C85F9551-61AC-4404-A2C5-61908D710298}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{628CA991-1E18-4032-819F-05FE5C7F6A77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="284">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="285">
   <si>
     <t>TC ID</t>
   </si>
@@ -103,9 +103,6 @@
     <t>Neg_0009</t>
   </si>
   <si>
-    <t>නෑ, මට දෙන්න බෑ.</t>
-  </si>
-  <si>
     <t>Responses</t>
   </si>
   <si>
@@ -595,12 +592,6 @@
     <t>සුභ නෙත් උදසනක්!</t>
   </si>
   <si>
-    <t>nae, mata denna ba.</t>
-  </si>
-  <si>
-    <t>නැ, මට දෙන්න බෑහ්.</t>
-  </si>
-  <si>
     <t>tika tika rudiraya galagena giya</t>
   </si>
   <si>
@@ -616,9 +607,6 @@
     <t>අද රෑ 10:45PM වෙනකොට අපේ පැවරුමේ මුල් කොටස ඉවර කරගන්න සෙට් එකටම zoom එන්න පුළුවන්ද?</t>
   </si>
   <si>
-    <t>අද රෑ 10:45PM වෙනකොට අපේ පවරුමේ මුල් කොටස ඉවර කරගන්න සෙට් එකටම zoom එන්න පුළුවන්ද?</t>
-  </si>
-  <si>
     <t>mn oyt passe anubawa karannam.</t>
   </si>
   <si>
@@ -658,96 +646,33 @@
     <t xml:space="preserve">පරිස්සමෙන් ගිහින් එන්න </t>
   </si>
   <si>
-    <t>machan, mama heta ude 8:30AM weddi SLIIT ekata enawa. ape project eke documentation tika PDF ekak widihata aran enna. eka table eka udin thiyanna amathaka karanna epa. nathnam apita ada wede iwara karanna bari wei. parissamen waren!</t>
-  </si>
-  <si>
-    <t>මට තවදුරටත් මේක ඉවසන්න බැහැ! වැඩේ හරියට කරන්න බැරි නම් අයින් වෙන්න 😅</t>
-  </si>
-  <si>
-    <t>මචං, මම හෙට උදේ 8:30AM වෙද්දී SLIIT එකට එනවා. අපේ project එකේ documentation ටික PDF එකක් විදිහට අරන් එන්න. ඒක table එක උඩින් තියන්න අමතක කරන්න එපා. නැත්නම් අපිට අද වැඩේ ඉවර කරන්න බැරි වෙයි. පරිස්සමෙන් වරෙන්!</t>
-  </si>
-  <si>
     <t>oya ticket eka book karada cheena maha prakareta?</t>
   </si>
   <si>
-    <t>mama ada office awe train eken nisa harima udyogimath.</t>
-  </si>
-  <si>
-    <t>මම අද office ආවේ train එකෙන් නිසා හරිම උද්‍යෝගිමත්.</t>
-  </si>
-  <si>
     <t>meeting එක 9:00AM කැන්ටිමේදී පටන් ගන්න කිව්වා.</t>
   </si>
   <si>
     <t>meeting eka 9:00AM kantimedi patan ganna kiwwa.</t>
   </si>
   <si>
-    <t>meeting එක 9:00AM කන්ටිමෙදි පටන් ගන්න කිව්වා.</t>
-  </si>
-  <si>
-    <t>ඔයා ටිකට් එක book කරාද චීන මහා ප්‍රකරෙට?</t>
-  </si>
-  <si>
     <t>ඔයා ticket එක book කරාද චීන මහා ප්‍රාකාරෙට?</t>
   </si>
   <si>
-    <t>මම අද office ආවේ train එකෙන් නිසා හරිම උද්යෝගීමාත්.</t>
-  </si>
-  <si>
-    <t>Dollar 2000 කින් එවුරෝෆේ ගිහින් එන්න පුළුවන්ද?</t>
-  </si>
-  <si>
-    <t>මේ link එක බලන්න: https://lk.නිවුස්</t>
-  </si>
-  <si>
-    <t>ado pattai bung, uba eka supiriyatama karala thiyenawa</t>
-  </si>
-  <si>
-    <t>අඩෝ පට්ටයි බං, උඹ ඒක සුපිරියටම කරලා තියෙනවා</t>
-  </si>
-  <si>
-    <t>අඩෝ පට්ටයි බුන්ග්, උඹ ඒක සුපිරියටම කරලා තියෙනවා</t>
-  </si>
-  <si>
-    <t>මචන් , මම හෙට උදේ 8:30AM වෙද්දී SLIIT එකට එනවා. අපේ project එකේ documentation ටික PDF එකක් විදිහට අරන් එන්න. ඒක table එක උඩින් තියන්න අමතක කරන්න එපා. නැත්නම් අපිට අද වැඩේ ඉවර කරන්න බැරි වෙයි. පරිස්සමෙන් වරෙන්!</t>
-  </si>
-  <si>
     <t>oya laga MID exam PDF eka thiyanawada?</t>
   </si>
   <si>
     <t>ඔයා ළඟ MID exam PDF එක තියෙනවාද?</t>
   </si>
   <si>
-    <t>ඔය ලඟ MID exam PDF එක තියෙනවාද?</t>
-  </si>
-  <si>
-    <t>Evidence: The system incorrectly splits and transliterate 'අර්යාශ්ඨාංගික මාර්ගය' and 'අවබෝද'.</t>
-  </si>
-  <si>
-    <t>Evidence:  'බැරෑරුම් ' is incorrectly transliterated as 'බාරරුම්' with an error.</t>
-  </si>
-  <si>
-    <t>Evidence: The command ' බං' is mangled as 'බුන්ග්'</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rationale: 'ප්‍රබන්ධ' is rendered as 'ප්රභාණ්ඩ' — a completely wrong transliteration . </t>
-  </si>
-  <si>
     <t>Rationale: 'උදෑසනක්!' should map correctly  but produces 'උදසනක්!' missing the aspiring marker.</t>
   </si>
   <si>
-    <t>Rationale: 'කලවැදි පැටියා' is distorted as 'කලවාදි පටිය'.</t>
-  </si>
-  <si>
     <t>Rationale: 'අයවැය file එකs' is stretched to 'අයවය file එක' by missing some parts of the letters.</t>
   </si>
   <si>
     <t xml:space="preserve">Evidence: Short polite request 'නැගිටිනකම්.' is mangled. </t>
   </si>
   <si>
-    <t>Evidence: 'බෑ.' is incorrectly split to ' බෑහ්.' — a strange -Sinhala character sequence.</t>
-  </si>
-  <si>
     <t>Evidence:  'නිවැරදි' is elongated incorrectly to 'නිවරදි'.</t>
   </si>
   <si>
@@ -757,15 +682,6 @@
     <t>හිත හැදෙන්නත් එක්ක හෙමින් හෙමින් ගියනම් මට හොඳයි වගේ.</t>
   </si>
   <si>
-    <t>Rationale: 'හැදෙන්නත් ' converted to 'හදෙන්නත්'</t>
-  </si>
-  <si>
-    <t>මම යනවා උද්‍යනයට.... ඔයත් එනවද අපි එක්ක?</t>
-  </si>
-  <si>
-    <t>Evidence: 'උද්‍යානයට.' is mangled to 'උද්‍යනයට.'. Punctuation disrupts phonetic parsing.</t>
-  </si>
-  <si>
     <t>Rationale: 'දෝලාවෙන්' becomes ' දූපාවෙන්' incorrectly</t>
   </si>
   <si>
@@ -778,33 +694,12 @@
     <t>Rationale: 'paris hotel ' is converted to 'පරිස් හොටෙල් ' .</t>
   </si>
   <si>
-    <t xml:space="preserve">Rationale: 'චීන මහා ප්‍රාකාරෙට?' is transliterated to 'චීන මහා ප්‍රකරෙට?' — incorrect sound based breakdown. </t>
-  </si>
-  <si>
-    <t>Evidence: 'උද්‍යෝගිමත්.' is mangled to 'උද්යෝගීමාත්.' System cannot preserve multi-word English phrases.</t>
-  </si>
-  <si>
-    <t>Rationale:  'soon එනවෝ' becomes 'soon එනවාඕ' with double vowel. .</t>
-  </si>
-  <si>
     <t xml:space="preserve">Evidence: 'අසල්වැසියන්' is transliterated to 'අසල්වාසියන් ' — incorrect sound based mapping that loses the recognised term. </t>
   </si>
   <si>
-    <t>Rationale: 'ලොකු නැන්දේ' is expanded to 'ලොකු නන්දේ' adding punctuation inside the shortened form.</t>
-  </si>
-  <si>
     <t>Evidence: 'කථිකාචාර්යවරයා' is mangled incorrectly</t>
   </si>
   <si>
-    <t>Rationale: 'මගේ පුතේ' produced as 'මගේ පුතී' — destroying the  name.</t>
-  </si>
-  <si>
-    <t>Rationale: 'ළමයි සේරටම' is expanded to 'ළමයි  සර්ට්ම' with dots between letters — incorrect .</t>
-  </si>
-  <si>
-    <t>Rationale:'ඔයා' converted to 'ඔය' incorrectly</t>
-  </si>
-  <si>
     <t>Rationale: 'lab' is converted as 'ලබ්' — wrong vowel and unusual Sinhala characters.Shortened English forms used in chat are broken.</t>
   </si>
   <si>
@@ -832,9 +727,6 @@
     <t xml:space="preserve">Rationale: 'භූගෝලය ' converted incorrectly as බූගෝලය </t>
   </si>
   <si>
-    <t xml:space="preserve">Rationale: 'Europe' is incorrectly converted as 'එවුරෝෆේ '. </t>
-  </si>
-  <si>
     <t xml:space="preserve">Rationale: 'කැන්ටිමේදී' is broken as 'කන්ටිමෙදි ' </t>
   </si>
   <si>
@@ -856,22 +748,133 @@
     <t xml:space="preserve">Rationale: Slang 'බං' becomes 'බුන්ග්' with excess vowels. </t>
   </si>
   <si>
-    <t>Rationale: 'https://lk.news' is partially transliterated to 'https://lk.නිවුස්'. The URL 'https://' is crushed'. URLs must be preserved directly.</t>
-  </si>
-  <si>
     <t>Rationale: 'support@company.com' becomes 'support@company.කොම්' destroying the recognised term.</t>
   </si>
   <si>
     <t>Rationale: Emoji is missing</t>
   </si>
   <si>
-    <t>Rationale: Long paragraph causes cascading transliteration  errors. 'machan' becomes 'මචන්'. Long inputs expose cumulative syntax error.</t>
-  </si>
-  <si>
-    <t>Rationale: Anger emoji turned into happy one .Error is there.</t>
-  </si>
-  <si>
-    <t>Rationale: 'පැවරුමේ' became 'පවරුමේ' .That's incorrect conversion</t>
+    <t>nae, mata denna ba mage nidanaya</t>
+  </si>
+  <si>
+    <t>නෑ , මට දෙන්න බෑ මගේ නිධානය</t>
+  </si>
+  <si>
+    <t>නැ, මට දෙන්න බෑ මගේ නිදනය</t>
+  </si>
+  <si>
+    <t>ඔය ticket එක book කරාද චීන මහා ප්රකාරෙට?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rationale: 'චීන මහා ප්‍රාකාරෙට?' is transliterated to 'චීන මහා ප්රකාරෙට?' — incorrect sound based breakdown. </t>
+  </si>
+  <si>
+    <t>mama ada office awe train eken nisa harima javasampanna bawak danenawa.</t>
+  </si>
+  <si>
+    <t>මම අද office ආවේ train එකෙන් නිසා හරිම ජවසම්පන්න බවක් දැනෙනවා.</t>
+  </si>
+  <si>
+    <t>මම අද office ආවේ train එකෙන් නිසා හරිම ජපකම්පන්න බවක් දැනෙනවා.</t>
+  </si>
+  <si>
+    <t>Evidence: 'ජවසම්පන්න.' is mangled to 'ජපකම්පන්න' System cannot preserve multi-word English phrases.</t>
+  </si>
+  <si>
+    <t>ඔය ළග MID exam PDF ඒක තියනවද?</t>
+  </si>
+  <si>
+    <t>Rationale:'ඔයා' converted to 'ඔය' and ' PDF එක' converted to ' PDF ඒක' incorrectly</t>
+  </si>
+  <si>
+    <t>dollar 2000 කින්‍යුරෝපය ගිහින් එන්න පුළුවන්ද?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rationale: 'Europe' is incorrectly converted as 'කින්‍යුරෝපය '. </t>
+  </si>
+  <si>
+    <t>meeting එක 9:00AM කන්ටිමේදි පටන් ගන්න කිව්වා.</t>
+  </si>
+  <si>
+    <t>ado pattai bung, ubanm real waddek</t>
+  </si>
+  <si>
+    <t>අඩො පට්ටයි බුන්ග්, උබ නම් real වද්දෙක්</t>
+  </si>
+  <si>
+    <t>අඩෝ පට්ටයි බං, උඹනම් real වැඩ්ඩෙක්</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rationale: Slang 'වැඩ්ඩෙක්' becomes 'වද්දෙක්' with excess vowels. </t>
+  </si>
+  <si>
+    <t>මේ link එක බලන්න: https://ලක්.news</t>
+  </si>
+  <si>
+    <t>Rationale: 'https://lk.news' is partially transliterated to ' https://ලක්.news'. The URL 'https://' is crushed'. URLs must be preserved directly.</t>
+  </si>
+  <si>
+    <t>Rationale: Long paragraph causes cascading transliteration  errors. 'පටස්ගාලා වරෙන්!' becomes 'පටස්ගල වරෙන්!'. Long inputs expose cumulative syntax error.</t>
+  </si>
+  <si>
+    <t>මම යනවා උද්යානයට... ඔයත් එනවද අපි එක්ක?</t>
+  </si>
+  <si>
+    <t>Rationale: 'ළමයි සේරටම' is expanded to 'ළමයි  සර්ට්ම' — incorrect .</t>
+  </si>
+  <si>
+    <t>මට තවදුරටත් මේක ඉවසන්න බැහැ! වැඩේ හරියට කරන්න බැරි නම් අයින් වෙන්න 🤣</t>
+  </si>
+  <si>
+    <t>Rationale: Anger emoji turned into 'haha' laughing face .Massive error is there.</t>
+  </si>
+  <si>
+    <t>අද රෑ 10:45PM වෙනකොට අපේ පවරුමේ මුල් කොටස ඉවර කරගන්න set එකටම zoom එන්න පුළුවන්ද?</t>
+  </si>
+  <si>
+    <t>Evidence: The system demonstrates severe phonetic mapping failure with complex religious/philosophical terms and fails to correctly render characters.The system incorrectly splits and transliterate 'අර්යාශ්ඨාංගික මාර්ගය' and 'අවබෝද'.</t>
+  </si>
+  <si>
+    <t>Evidence: Phonetic inaccuracy in mapping vowel length (Vowel Elongation), where the specific term  'බැරෑරුම් ' is incorrectly transliterated as 'බාරරුම්' with an error.</t>
+  </si>
+  <si>
+    <t>Evidence: Failure in handling colloquial slang/particles.The word ' බං' is mangled as 'බුන්ග්'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rationale:The system incorrectly processes combined consonants. 'ප්‍රබන්ධ' is rendered as 'ප්රභාණ්ඩ' — a completely wrong transliteration . </t>
+  </si>
+  <si>
+    <t>Rationale: 'කලවැදි පැටියා' is distorted as 'කලවාදි පටිය' which changes the intended meaning.</t>
+  </si>
+  <si>
+    <t>Evidence: 'නිධානය' is incorrectly split to '  නිදනය' — a strange -Sinhala character sequence.</t>
+  </si>
+  <si>
+    <t>Rationale: 'හැදෙන්නත් ' converted to 'හදෙන්නත්' leading to a loss of the intended emotional tone due to over elongation of following vowels.</t>
+  </si>
+  <si>
+    <t>Evidence: 'උද්‍යානයට.' is mangled to 'උද්යානයට'. Punctuation disrupts phonetic parsing.The system struggles with the 'Yansaya' character in proper nouns or technical terms, resulting in broken character rendering.</t>
+  </si>
+  <si>
+    <t>Rationale:  'soon එනවෝ' becomes 'soon එනවාඕ' .Demonstrates poor handling of imperative forms</t>
+  </si>
+  <si>
+    <t>Rationale: 'මගේ පුතේ' produced as 'මගේ පුතී' — The system demonstrates a lack of contextual awareness, incorrectly transliterating proper nouns as common nouns with elongated vowels.</t>
+  </si>
+  <si>
+    <t>Rationale: 'පැවරුමේ' became 'පවරුමේ' .That's incorrect conversion.The system demonstrates a 'Contextual Gap' by failing to recognize common university related terms used by students.</t>
+  </si>
+  <si>
+    <t>Rationale: 'ලොකු නැන්දේ' is expanded to 'ලොකු නන්දේ' adding no meaning to the sentence.</t>
+  </si>
+  <si>
+    <t>machan, mama heta ude 8:30AM weddi SLIIT ekata enawa. ape project eke documentation tika PDF ekak widihata aran enna campus library eka gawata. Eekarala eeka table eka udin thiyanna amathaka karanna epa.Yathura LIC gawa athi, nathnam apita ada dawasa athulatha wede iwara karanna bari wei. patasgala waren eenisa bus eke hari</t>
+  </si>
+  <si>
+    <t>මචං, මම හෙට උදේ 8:30AM වෙද්දී SLIIT එකට එනවා. අපේ project එකේ documentation ටික PDF එකක් විදිහට අරන් එන්න කැම්පස් library එක ගාවට. ඒකරලා ඒක ටේබල් එක උඩින් තියන්න අමතක කරන්න එපා. යතුර LIC ගාව ඇති, නැත්නම් අපිට අද දවස ඇතුළත වැඩේ ඉවර කරන්න බැරි වෙයි. පටස්ගාලා වරෙන් ඒනිසා bus එකේ හරි</t>
+  </si>
+  <si>
+    <t>මචං, මම හෙට උදේ 8:30AM වෙද්දී SLIIT එකට එනවා. අපේ project එකේ documentation ටික PDF එකක් විදිහට අරන් එන්න කැම්පස් library එක ගාවට. ඒකරලා ඒක ටේබල් එක උඩින් තියන්න අමතක කරන්න එපා. යතුර LIC ගාව ඇති, නැත්නම් අපිට අද දවස ඇතුළත වැඩේ ඉවර කරන්න බැරි වෙයි. පටස්ගල වරෙන් ඒනිසා bus එකේ හරි</t>
   </si>
 </sst>
 </file>
@@ -1308,13 +1311,13 @@
         <v>13</v>
       </c>
       <c r="C2" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="D2" s="3" t="s">
         <v>185</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="E2" s="3" t="s">
         <v>186</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>187</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>10</v>
@@ -1323,7 +1326,7 @@
         <v>11</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>233</v>
+        <v>270</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="49.95" customHeight="1">
@@ -1334,13 +1337,13 @@
         <v>13</v>
       </c>
       <c r="C3" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="E3" s="3" t="s">
         <v>126</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>125</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>127</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>10</v>
@@ -1349,7 +1352,7 @@
         <v>11</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>234</v>
+        <v>271</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="49.95" customHeight="1">
@@ -1366,7 +1369,7 @@
         <v>16</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>10</v>
@@ -1375,7 +1378,7 @@
         <v>17</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>235</v>
+        <v>272</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="49.95" customHeight="1">
@@ -1386,13 +1389,13 @@
         <v>13</v>
       </c>
       <c r="C5" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="D5" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="E5" s="3" t="s">
         <v>123</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>124</v>
       </c>
       <c r="F5" s="2" t="s">
         <v>10</v>
@@ -1401,7 +1404,7 @@
         <v>17</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>236</v>
+        <v>273</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="49.95" customHeight="1">
@@ -1412,13 +1415,13 @@
         <v>9</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>20</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="F6" s="2" t="s">
         <v>10</v>
@@ -1427,7 +1430,7 @@
         <v>21</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>237</v>
+        <v>214</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="49.95" customHeight="1">
@@ -1438,13 +1441,13 @@
         <v>13</v>
       </c>
       <c r="C7" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="D7" s="3" t="s">
         <v>119</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="E7" s="3" t="s">
         <v>120</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>121</v>
       </c>
       <c r="F7" s="2" t="s">
         <v>10</v>
@@ -1453,7 +1456,7 @@
         <v>21</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>238</v>
+        <v>274</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="49.95" customHeight="1">
@@ -1464,13 +1467,13 @@
         <v>13</v>
       </c>
       <c r="C8" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D8" s="3" t="s">
         <v>116</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="E8" s="3" t="s">
         <v>117</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>118</v>
       </c>
       <c r="F8" s="2" t="s">
         <v>10</v>
@@ -1479,7 +1482,7 @@
         <v>24</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>239</v>
+        <v>215</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="49.95" customHeight="1">
@@ -1490,13 +1493,13 @@
         <v>9</v>
       </c>
       <c r="C9" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="D9" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="E9" s="2" t="s">
         <v>114</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>115</v>
       </c>
       <c r="F9" s="2" t="s">
         <v>10</v>
@@ -1505,7 +1508,7 @@
         <v>24</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>240</v>
+        <v>216</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="49.95" customHeight="1">
@@ -1516,1088 +1519,1088 @@
         <v>9</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>191</v>
+        <v>244</v>
       </c>
       <c r="D10" s="3" t="s">
+        <v>245</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>246</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G10" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="E10" s="3" t="s">
-        <v>192</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="G10" s="2" t="s">
-        <v>28</v>
-      </c>
       <c r="H10" s="5" t="s">
-        <v>241</v>
+        <v>275</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="49.95" customHeight="1">
       <c r="A11" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>13</v>
       </c>
       <c r="C11" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="D11" s="3" t="s">
         <v>110</v>
       </c>
-      <c r="D11" s="3" t="s">
+      <c r="E11" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="E11" s="3" t="s">
-        <v>112</v>
-      </c>
       <c r="F11" s="2" t="s">
         <v>10</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>242</v>
+        <v>217</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="49.95" customHeight="1">
       <c r="A12" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>9</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="F12" s="2" t="s">
         <v>10</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>243</v>
+        <v>218</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="49.95" customHeight="1">
       <c r="A13" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>13</v>
       </c>
       <c r="C13" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="E13" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="D13" s="3" t="s">
-        <v>244</v>
-      </c>
-      <c r="E13" s="3" t="s">
-        <v>109</v>
-      </c>
       <c r="F13" s="2" t="s">
         <v>10</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>245</v>
+        <v>276</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="49.95" customHeight="1">
       <c r="A14" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>265</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G14" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="B14" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="D14" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="E14" s="3" t="s">
-        <v>246</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="G14" s="2" t="s">
-        <v>34</v>
-      </c>
       <c r="H14" s="3" t="s">
-        <v>247</v>
+        <v>277</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="49.95" customHeight="1">
       <c r="A15" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>9</v>
       </c>
       <c r="C15" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="D15" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="D15" s="3" t="s">
+      <c r="E15" s="3" t="s">
         <v>104</v>
       </c>
-      <c r="E15" s="3" t="s">
-        <v>105</v>
-      </c>
       <c r="F15" s="2" t="s">
         <v>10</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>248</v>
+        <v>220</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="49.95" customHeight="1">
       <c r="A16" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>9</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="F16" s="2" t="s">
         <v>10</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H16" s="3" t="s">
-        <v>249</v>
+        <v>221</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="49.95" customHeight="1">
       <c r="A17" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>13</v>
       </c>
       <c r="C17" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="E17" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="D17" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="E17" s="3" t="s">
-        <v>101</v>
-      </c>
       <c r="F17" s="2" t="s">
         <v>10</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H17" s="3" t="s">
-        <v>250</v>
+        <v>222</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="49.95" customHeight="1">
       <c r="A18" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G18" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="B18" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="D18" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="E18" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="F18" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="G18" s="2" t="s">
-        <v>40</v>
-      </c>
       <c r="H18" s="5" t="s">
-        <v>251</v>
+        <v>223</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="49.95" customHeight="1">
       <c r="A19" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>9</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>215</v>
+        <v>208</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>222</v>
+        <v>211</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>221</v>
+        <v>247</v>
       </c>
       <c r="F19" s="2" t="s">
         <v>10</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="H19" s="5" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
     </row>
     <row r="20" spans="1:8" ht="49.95" customHeight="1">
       <c r="A20" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>250</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G20" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B20" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C20" s="3" t="s">
-        <v>216</v>
-      </c>
-      <c r="D20" s="3" t="s">
-        <v>217</v>
-      </c>
-      <c r="E20" s="3" t="s">
-        <v>223</v>
-      </c>
-      <c r="F20" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="G20" s="2" t="s">
-        <v>43</v>
-      </c>
       <c r="H20" s="5" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="49.95" customHeight="1">
       <c r="A21" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B21" s="2" t="s">
         <v>13</v>
       </c>
       <c r="C21" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>183</v>
+      </c>
+      <c r="E21" s="3" t="s">
         <v>182</v>
       </c>
-      <c r="D21" s="3" t="s">
-        <v>184</v>
-      </c>
-      <c r="E21" s="3" t="s">
-        <v>183</v>
-      </c>
       <c r="F21" s="2" t="s">
         <v>10</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="H21" s="5" t="s">
-        <v>254</v>
+        <v>278</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="49.95" customHeight="1">
       <c r="A22" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="E22" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="F22" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G22" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="B22" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="D22" s="3" t="s">
-        <v>95</v>
-      </c>
-      <c r="E22" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="F22" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="G22" s="2" t="s">
-        <v>46</v>
-      </c>
       <c r="H22" s="5" t="s">
-        <v>255</v>
+        <v>224</v>
       </c>
     </row>
     <row r="23" spans="1:8" ht="49.95" customHeight="1">
       <c r="A23" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B23" s="2" t="s">
         <v>13</v>
       </c>
       <c r="C23" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="D23" s="3" t="s">
         <v>179</v>
       </c>
-      <c r="D23" s="3" t="s">
+      <c r="E23" s="3" t="s">
         <v>180</v>
       </c>
-      <c r="E23" s="3" t="s">
-        <v>181</v>
-      </c>
       <c r="F23" s="2" t="s">
         <v>10</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H23" s="5" t="s">
-        <v>256</v>
+        <v>281</v>
       </c>
     </row>
     <row r="24" spans="1:8" ht="49.95" customHeight="1">
       <c r="A24" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G24" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="B24" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="D24" s="3" t="s">
-        <v>178</v>
-      </c>
-      <c r="E24" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="F24" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="G24" s="2" t="s">
-        <v>49</v>
-      </c>
       <c r="H24" s="5" t="s">
-        <v>257</v>
+        <v>225</v>
       </c>
     </row>
     <row r="25" spans="1:8" ht="49.95" customHeight="1">
       <c r="A25" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B25" s="2" t="s">
         <v>13</v>
       </c>
       <c r="C25" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E25" s="3" t="s">
         <v>173</v>
       </c>
-      <c r="D25" s="3" t="s">
-        <v>175</v>
-      </c>
-      <c r="E25" s="3" t="s">
-        <v>174</v>
-      </c>
       <c r="F25" s="2" t="s">
         <v>10</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="H25" s="5" t="s">
-        <v>258</v>
+        <v>279</v>
       </c>
     </row>
     <row r="26" spans="1:8" ht="49.95" customHeight="1">
       <c r="A26" s="2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B26" s="2" t="s">
         <v>13</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D26" s="3" t="s">
         <v>171</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="F26" s="2" t="s">
         <v>10</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="H26" s="5" t="s">
-        <v>259</v>
+        <v>266</v>
       </c>
     </row>
     <row r="27" spans="1:8" ht="49.95" customHeight="1">
       <c r="A27" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B27" s="2" t="s">
         <v>9</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>230</v>
+        <v>212</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>231</v>
+        <v>213</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>232</v>
+        <v>253</v>
       </c>
       <c r="F27" s="2" t="s">
         <v>10</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="H27" s="5" t="s">
-        <v>260</v>
+        <v>254</v>
       </c>
     </row>
     <row r="28" spans="1:8" ht="49.95" customHeight="1">
       <c r="A28" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="D28" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="E28" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="F28" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G28" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="B28" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C28" s="3" t="s">
-        <v>166</v>
-      </c>
-      <c r="D28" s="3" t="s">
-        <v>167</v>
-      </c>
-      <c r="E28" s="3" t="s">
-        <v>168</v>
-      </c>
-      <c r="F28" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="G28" s="2" t="s">
-        <v>55</v>
-      </c>
       <c r="H28" s="5" t="s">
-        <v>261</v>
+        <v>226</v>
       </c>
     </row>
     <row r="29" spans="1:8" ht="49.95" customHeight="1">
       <c r="A29" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B29" s="2" t="s">
         <v>9</v>
       </c>
       <c r="C29" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D29" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="D29" s="3" t="s">
-        <v>58</v>
-      </c>
       <c r="E29" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="F29" s="2" t="s">
         <v>10</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="H29" s="3" t="s">
-        <v>262</v>
+        <v>227</v>
       </c>
     </row>
     <row r="30" spans="1:8" ht="49.95" customHeight="1">
       <c r="A30" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="D30" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="E30" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="F30" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G30" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="B30" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C30" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="D30" s="3" t="s">
-        <v>165</v>
-      </c>
-      <c r="E30" s="3" t="s">
-        <v>164</v>
-      </c>
-      <c r="F30" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="G30" s="2" t="s">
-        <v>60</v>
-      </c>
       <c r="H30" s="5" t="s">
-        <v>263</v>
+        <v>228</v>
       </c>
     </row>
     <row r="31" spans="1:8" ht="49.95" customHeight="1">
       <c r="A31" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B31" s="2" t="s">
         <v>13</v>
       </c>
       <c r="C31" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="D31" s="2" t="s">
         <v>160</v>
       </c>
-      <c r="D31" s="2" t="s">
+      <c r="E31" s="3" t="s">
         <v>161</v>
       </c>
-      <c r="E31" s="3" t="s">
-        <v>162</v>
-      </c>
       <c r="F31" s="2" t="s">
         <v>10</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="H31" s="5" t="s">
-        <v>264</v>
+        <v>229</v>
       </c>
     </row>
     <row r="32" spans="1:8" ht="49.95" customHeight="1">
       <c r="A32" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="D32" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="E32" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="F32" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G32" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="B32" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C32" s="2" t="s">
-        <v>157</v>
-      </c>
-      <c r="D32" s="3" t="s">
-        <v>158</v>
-      </c>
-      <c r="E32" s="3" t="s">
-        <v>159</v>
-      </c>
-      <c r="F32" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="G32" s="2" t="s">
-        <v>63</v>
-      </c>
       <c r="H32" s="5" t="s">
-        <v>265</v>
+        <v>230</v>
       </c>
     </row>
     <row r="33" spans="1:8" ht="49.95" customHeight="1">
       <c r="A33" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="C33" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="D33" s="3" t="s">
         <v>154</v>
       </c>
-      <c r="D33" s="3" t="s">
+      <c r="E33" s="3" t="s">
         <v>155</v>
       </c>
-      <c r="E33" s="3" t="s">
-        <v>156</v>
-      </c>
       <c r="F33" s="2" t="s">
         <v>10</v>
       </c>
       <c r="G33" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="H33" s="5" t="s">
-        <v>266</v>
+        <v>231</v>
       </c>
     </row>
     <row r="34" spans="1:8" ht="49.95" customHeight="1">
       <c r="A34" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C34" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="D34" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="E34" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="F34" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G34" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="B34" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C34" s="3" t="s">
-        <v>151</v>
-      </c>
-      <c r="D34" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="E34" s="3" t="s">
-        <v>152</v>
-      </c>
-      <c r="F34" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="G34" s="2" t="s">
-        <v>66</v>
-      </c>
       <c r="H34" s="3" t="s">
-        <v>267</v>
+        <v>232</v>
       </c>
     </row>
     <row r="35" spans="1:8" ht="49.95" customHeight="1">
       <c r="A35" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="C35" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="D35" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="D35" s="2" t="s">
-        <v>150</v>
-      </c>
       <c r="E35" s="3" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="F35" s="2" t="s">
         <v>10</v>
       </c>
       <c r="G35" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="H35" s="3" t="s">
-        <v>268</v>
+        <v>233</v>
       </c>
     </row>
     <row r="36" spans="1:8" ht="49.95" customHeight="1">
       <c r="A36" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B36" s="2" t="s">
         <v>9</v>
       </c>
       <c r="C36" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="D36" s="3" t="s">
         <v>146</v>
       </c>
-      <c r="D36" s="3" t="s">
+      <c r="E36" s="3" t="s">
         <v>147</v>
       </c>
-      <c r="E36" s="3" t="s">
-        <v>148</v>
-      </c>
       <c r="F36" s="2" t="s">
         <v>10</v>
       </c>
       <c r="G36" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="H36" s="3" t="s">
-        <v>269</v>
+        <v>234</v>
       </c>
     </row>
     <row r="37" spans="1:8" ht="49.95" customHeight="1">
       <c r="A37" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B37" s="2" t="s">
         <v>13</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>224</v>
+        <v>255</v>
       </c>
       <c r="F37" s="2" t="s">
         <v>10</v>
       </c>
       <c r="G37" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="H37" s="5" t="s">
-        <v>270</v>
+        <v>256</v>
       </c>
     </row>
     <row r="38" spans="1:8" ht="49.95" customHeight="1">
       <c r="A38" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C38" s="3" t="s">
+        <v>210</v>
+      </c>
+      <c r="D38" s="3" t="s">
+        <v>209</v>
+      </c>
+      <c r="E38" s="3" t="s">
+        <v>257</v>
+      </c>
+      <c r="F38" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G38" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="B38" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C38" s="3" t="s">
-        <v>219</v>
-      </c>
-      <c r="D38" s="3" t="s">
-        <v>218</v>
-      </c>
-      <c r="E38" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="F38" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="G38" s="2" t="s">
-        <v>72</v>
-      </c>
       <c r="H38" s="5" t="s">
-        <v>271</v>
+        <v>235</v>
       </c>
     </row>
     <row r="39" spans="1:8" ht="49.95" customHeight="1">
       <c r="A39" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B39" s="2" t="s">
         <v>13</v>
       </c>
       <c r="C39" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="D39" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="E39" s="3" t="s">
         <v>144</v>
       </c>
-      <c r="D39" s="3" t="s">
-        <v>143</v>
-      </c>
-      <c r="E39" s="3" t="s">
-        <v>145</v>
-      </c>
       <c r="F39" s="2" t="s">
         <v>10</v>
       </c>
       <c r="G39" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="H39" s="5" t="s">
-        <v>272</v>
+        <v>236</v>
       </c>
     </row>
     <row r="40" spans="1:8" ht="49.95" customHeight="1">
       <c r="A40" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D40" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="E40" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="F40" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G40" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="B40" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C40" s="2" t="s">
-        <v>140</v>
-      </c>
-      <c r="D40" s="3" t="s">
-        <v>141</v>
-      </c>
-      <c r="E40" s="3" t="s">
-        <v>142</v>
-      </c>
-      <c r="F40" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="G40" s="2" t="s">
-        <v>75</v>
-      </c>
       <c r="H40" s="3" t="s">
-        <v>273</v>
+        <v>237</v>
       </c>
     </row>
     <row r="41" spans="1:8" ht="49.95" customHeight="1">
       <c r="A41" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B41" s="2" t="s">
         <v>13</v>
       </c>
       <c r="C41" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="D41" s="3" t="s">
         <v>137</v>
       </c>
-      <c r="D41" s="3" t="s">
+      <c r="E41" s="3" t="s">
         <v>138</v>
       </c>
-      <c r="E41" s="3" t="s">
-        <v>139</v>
-      </c>
       <c r="F41" s="2" t="s">
         <v>10</v>
       </c>
       <c r="G41" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H41" s="5" t="s">
-        <v>274</v>
+        <v>238</v>
       </c>
     </row>
     <row r="42" spans="1:8" ht="49.95" customHeight="1">
       <c r="A42" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="D42" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="E42" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="F42" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G42" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="B42" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C42" s="2" t="s">
-        <v>134</v>
-      </c>
-      <c r="D42" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="E42" s="3" t="s">
-        <v>136</v>
-      </c>
-      <c r="F42" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="G42" s="2" t="s">
-        <v>78</v>
-      </c>
       <c r="H42" s="5" t="s">
-        <v>275</v>
+        <v>239</v>
       </c>
     </row>
     <row r="43" spans="1:8" ht="49.95" customHeight="1">
       <c r="A43" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="C43" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="D43" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="E43" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="D43" s="3" t="s">
-        <v>133</v>
-      </c>
-      <c r="E43" s="3" t="s">
-        <v>132</v>
-      </c>
       <c r="F43" s="2" t="s">
         <v>10</v>
       </c>
       <c r="G43" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H43" s="5" t="s">
-        <v>276</v>
+        <v>240</v>
       </c>
     </row>
     <row r="44" spans="1:8" ht="49.95" customHeight="1">
       <c r="A44" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C44" s="3" t="s">
+        <v>258</v>
+      </c>
+      <c r="D44" s="3" t="s">
+        <v>260</v>
+      </c>
+      <c r="E44" s="3" t="s">
+        <v>259</v>
+      </c>
+      <c r="F44" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G44" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="B44" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C44" s="3" t="s">
-        <v>226</v>
-      </c>
-      <c r="D44" s="3" t="s">
-        <v>227</v>
-      </c>
-      <c r="E44" s="3" t="s">
-        <v>228</v>
-      </c>
-      <c r="F44" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="G44" s="2" t="s">
-        <v>81</v>
-      </c>
       <c r="H44" s="3" t="s">
-        <v>277</v>
+        <v>261</v>
       </c>
     </row>
     <row r="45" spans="1:8" ht="49.95" customHeight="1">
       <c r="A45" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B45" s="2" t="s">
         <v>13</v>
       </c>
       <c r="C45" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="D45" s="3" t="s">
         <v>128</v>
       </c>
-      <c r="D45" s="3" t="s">
+      <c r="E45" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="E45" s="3" t="s">
-        <v>130</v>
-      </c>
       <c r="F45" s="2" t="s">
         <v>10</v>
       </c>
       <c r="G45" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="H45" s="5" t="s">
-        <v>277</v>
+        <v>241</v>
       </c>
     </row>
     <row r="46" spans="1:8" ht="49.95" customHeight="1">
       <c r="A46" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C46" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="B46" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C46" s="2" t="s">
+      <c r="D46" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="D46" s="3" t="s">
+      <c r="E46" s="3" t="s">
+        <v>262</v>
+      </c>
+      <c r="F46" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G46" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="E46" s="3" t="s">
-        <v>225</v>
-      </c>
-      <c r="F46" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="G46" s="2" t="s">
-        <v>86</v>
-      </c>
       <c r="H46" s="5" t="s">
-        <v>278</v>
+        <v>263</v>
       </c>
     </row>
     <row r="47" spans="1:8" ht="49.95" customHeight="1">
       <c r="A47" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B47" s="2" t="s">
         <v>13</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="D47" s="3" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="E47" s="3" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="F47" s="2" t="s">
         <v>10</v>
       </c>
       <c r="G47" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H47" s="5" t="s">
-        <v>279</v>
+        <v>242</v>
       </c>
     </row>
     <row r="48" spans="1:8" ht="49.95" customHeight="1">
       <c r="A48" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C48" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="D48" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="E48" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="F48" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G48" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="B48" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C48" s="2" t="s">
-        <v>208</v>
-      </c>
-      <c r="D48" s="2" t="s">
-        <v>207</v>
-      </c>
-      <c r="E48" s="2" t="s">
-        <v>213</v>
-      </c>
-      <c r="F48" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="G48" s="2" t="s">
-        <v>89</v>
-      </c>
       <c r="H48" s="5" t="s">
-        <v>282</v>
+        <v>268</v>
       </c>
     </row>
     <row r="49" spans="1:8" ht="49.95" customHeight="1">
       <c r="A49" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B49" s="2" t="s">
         <v>9</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="E49" s="3" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="F49" s="2" t="s">
         <v>10</v>
       </c>
       <c r="G49" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="H49" s="5" t="s">
-        <v>280</v>
+        <v>243</v>
       </c>
     </row>
     <row r="50" spans="1:8" ht="49.95" customHeight="1">
       <c r="A50" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="B50" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="B50" s="2" t="s">
-        <v>92</v>
-      </c>
       <c r="C50" s="3" t="s">
-        <v>212</v>
+        <v>282</v>
       </c>
       <c r="D50" s="3" t="s">
-        <v>214</v>
+        <v>283</v>
       </c>
       <c r="E50" s="3" t="s">
-        <v>229</v>
+        <v>284</v>
       </c>
       <c r="F50" s="2" t="s">
         <v>10</v>
       </c>
       <c r="G50" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="H50" s="3" t="s">
-        <v>281</v>
+        <v>264</v>
       </c>
     </row>
     <row r="51" spans="1:8" ht="49.95" customHeight="1">
       <c r="A51" s="2" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B51" s="2" t="s">
         <v>13</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="E51" s="3" t="s">
-        <v>198</v>
+        <v>269</v>
       </c>
       <c r="F51" s="2" t="s">
         <v>10</v>
       </c>
       <c r="G51" s="3" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H51" s="3" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
     </row>
   </sheetData>

</xml_diff>